<commit_message>
CAD3: displacement_auger, traction_compacting_tool and vibratory_displacement_tool move from equipmentClass to cuttingToolType; terminationOutcome gains stopped_short
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/cuttingToolType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/cuttingToolType.xlsx
@@ -1295,8 +1295,21 @@
         <f>IF(ISNA(VLOOKUP(B9,AssociatedElements!B$2:B2947,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>traction_compacting_tool</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Traction compacting tool</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>A displacement tool that advances by traction and compacts soil on both insertion and extraction, typically about half on each. Offered by Keller / Hayward Baker as an alternative to a single-pass displacement auger.</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="n"/>
       <c r="G9" s="9" t="n"/>
     </row>
@@ -1305,9 +1318,21 @@
         <f>IF(ISNA(VLOOKUP(B10,AssociatedElements!B$2:B2948,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="14" t="n"/>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>vibratory_displacement_tool</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Vibratory displacement tool</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>A displacement tool advanced by vibration rather than by rotary drilling or static push.</t>
+        </is>
+      </c>
       <c r="E10" s="13" t="n"/>
       <c r="F10" s="13" t="n"/>
       <c r="G10" s="9" t="n"/>
@@ -1640,7 +1665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -1788,14 +1813,32 @@
         <f>IF(ISNA(VLOOKUP(B9,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>traction_compacting_tool</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>//diggs:CuttingTool/diggs:toolType</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
         <f>IF(ISNA(VLOOKUP(B10,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B10" s="20" t="n"/>
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>vibratory_displacement_tool</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>//diggs:CuttingTool/diggs:toolType</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11">

</xml_diff>